<commit_message>
Add YelanTranquil --> Yelan remap
- Does require some Texture coordinate UV mapping
- Needed combine of VB part files and edit to corresponding indices
of Ib files
</commit_message>
<xml_diff>
--- a/Data/RemapDrafts/JeanRemapDraft.xlsx
+++ b/Data/RemapDrafts/JeanRemapDraft.xlsx
@@ -79,11 +79,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -504,10 +505,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="14.453125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="68" bestFit="1" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -531,9 +532,17 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>🦴🧭 The Vertex Group Cartographer: The 32nd member of The Council</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>